<commit_message>
v2.3: add progress bar + per-step verification to main.py pipeline
</commit_message>
<xml_diff>
--- a/data/Object-Models-Updated - only.xlsx
+++ b/data/Object-Models-Updated - only.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P93"/>
+  <dimension ref="A1:P96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5832,6 +5832,220 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>GPT-5.5</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/gpt-5.5</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>1000k上下文；顶级推理能力；高端定价</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>国外</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>闭源</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/gpt-5.5-pro</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>1000k上下文；高端定价</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Qwen3.6-27B</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Alibaba Cloud / Qwen Team</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>开源</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>28B</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>多模态</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>通用对话</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>https://llm-stats.com/models/qwen3.6-27b</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>强推理能力；顶级编码能力；Apache 2.0</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>llm-stats.com 排行榜 · HuggingFace 需登录(alibaba-cloud-/Qwen3.6-27B)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>